<commit_message>
Fix critical bug: Add medicine IDs and API endpoint to fix production DB
</commit_message>
<xml_diff>
--- a/backend/data/medicines.xlsx
+++ b/backend/data/medicines.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,9 @@
       <c r="I1" t="str">
         <v>image_url</v>
       </c>
+      <c r="J1" t="str">
+        <v>medicine_id</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,6 +459,9 @@
       <c r="I2" t="str">
         <v>https://images.unsplash.com/photo-1584308666744-24d5c474f2ae?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J2" t="str">
+        <v>f91d827d-a1e4-4df1-bbee-b4bba62b670b</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -485,6 +491,9 @@
       <c r="I3" t="str">
         <v>https://images.unsplash.com/photo-1471864190281-a93a3070b6de?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J3" t="str">
+        <v>317cb851-5cd6-4f85-a677-d2efa7518e1c</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -514,6 +523,9 @@
       <c r="I4" t="str">
         <v>https://images.unsplash.com/photo-1587854692152-cbe660dbde88?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J4" t="str">
+        <v>09b964d5-312c-40d7-b8e1-7b60c65ae2ed</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -543,6 +555,9 @@
       <c r="I5" t="str">
         <v>https://images.unsplash.com/photo-1550572017-4a6c5d8f2f8e?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J5" t="str">
+        <v>c0cb0270-a8f2-49e2-9c06-c6d5ba1dd0ff</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -572,6 +587,9 @@
       <c r="I6" t="str">
         <v>https://images.unsplash.com/photo-1584308666744-24d5c474f2ae?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J6" t="str">
+        <v>363eb244-ecd4-4433-b488-ceb63514dd15</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -601,6 +619,9 @@
       <c r="I7" t="str">
         <v>https://images.unsplash.com/photo-1471864190281-a93a3070b6de?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J7" t="str">
+        <v>61b93d7b-3a82-4fd7-b02b-62ae7a2d5c66</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -630,6 +651,9 @@
       <c r="I8" t="str">
         <v>https://images.unsplash.com/photo-1550572017-4a6c5d8f2f8e?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J8" t="str">
+        <v>417c05f6-90e5-4b73-8d6b-ddee18debf82</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -659,6 +683,9 @@
       <c r="I9" t="str">
         <v>https://images.unsplash.com/photo-1587854692152-cbe660dbde88?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J9" t="str">
+        <v>61337f17-bd59-40f8-81ea-6962853fa0c9</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -688,6 +715,9 @@
       <c r="I10" t="str">
         <v>https://images.unsplash.com/photo-1584308666744-24d5c474f2ae?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J10" t="str">
+        <v>8af29fb7-8c13-4e0c-bc71-53401d144bb2</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -717,6 +747,9 @@
       <c r="I11" t="str">
         <v>https://images.unsplash.com/photo-1471864190281-a93a3070b6de?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J11" t="str">
+        <v>281cea73-549d-4b2f-bbbd-f488520894de</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -746,6 +779,9 @@
       <c r="I12" t="str">
         <v>https://images.unsplash.com/photo-1550572017-4a6c5d8f2f8e?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J12" t="str">
+        <v>489369ab-0f7f-4bfd-a669-4896f65e83c8</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -775,10 +811,13 @@
       <c r="I13" t="str">
         <v>https://images.unsplash.com/photo-1587854692152-cbe660dbde88?w=400&amp;h=400&amp;fit=crop</v>
       </c>
+      <c r="J13" t="str">
+        <v>4ff62add-0ca9-4428-a449-f058fc404169</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>